<commit_message>
Refactor GLCodeHelper: migrate getLedgerOptions and getFundOptions methods to class methods and remove standalone functions
</commit_message>
<xml_diff>
--- a/sfdemosite-Extracted-GLCode.xlsx
+++ b/sfdemosite-Extracted-GLCode.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://parentpay-my.sharepoint.com/personal/pruthviraj_pardeshi_parentpay_com/Documents/Documents/Repos/playwright-SIMS-Finance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_56E7000DE1693B66C66002EFC8579551A12C6C36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5632E979-C2F9-4D81-B498-08EC95BA011A}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_56E7000DE1693B66C66002EFC8579551A12C6C36" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{264DA2C4-C48A-4255-9353-142076255F32}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2280" yWindow="2280" windowWidth="14400" windowHeight="7360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025-07-15" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="102">
   <si>
     <t>Cost Centre Code</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>Year 7 catch up grant</t>
-  </si>
-  <si>
-    <t>00002</t>
   </si>
   <si>
     <t>Pupil Premium</t>
@@ -737,8 +734,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -937,549 +934,549 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>30</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" t="s">
-        <v>32</v>
-      </c>
       <c r="E12" t="s">
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
         <v>33</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>34</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>35</v>
       </c>
-      <c r="D13" t="s">
-        <v>36</v>
-      </c>
       <c r="E13" t="s">
         <v>10</v>
       </c>
       <c r="F13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
         <v>33</v>
       </c>
-      <c r="B14" t="s">
-        <v>34</v>
-      </c>
       <c r="C14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" t="s">
         <v>37</v>
       </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
       <c r="E14" t="s">
         <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
       <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" t="s">
         <v>39</v>
       </c>
-      <c r="D15" t="s">
-        <v>40</v>
-      </c>
       <c r="E15" t="s">
         <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
         <v>33</v>
       </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
       <c r="C16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
         <v>41</v>
       </c>
-      <c r="D16" t="s">
-        <v>42</v>
-      </c>
       <c r="E16" t="s">
         <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
         <v>33</v>
       </c>
-      <c r="B17" t="s">
-        <v>34</v>
-      </c>
       <c r="C17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" t="s">
         <v>43</v>
       </c>
-      <c r="D17" t="s">
-        <v>44</v>
-      </c>
       <c r="E17" t="s">
         <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
         <v>33</v>
       </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
       <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
         <v>45</v>
       </c>
-      <c r="D18" t="s">
-        <v>46</v>
-      </c>
       <c r="E18" t="s">
         <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
         <v>33</v>
       </c>
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
       <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
         <v>47</v>
       </c>
-      <c r="D19" t="s">
-        <v>48</v>
-      </c>
       <c r="E19" t="s">
         <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
         <v>33</v>
       </c>
-      <c r="B20" t="s">
-        <v>34</v>
-      </c>
       <c r="C20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" t="s">
         <v>49</v>
       </c>
-      <c r="D20" t="s">
-        <v>50</v>
-      </c>
       <c r="E20" t="s">
         <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" t="s">
         <v>51</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>52</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>53</v>
       </c>
-      <c r="D21" t="s">
-        <v>54</v>
-      </c>
       <c r="E21" t="s">
         <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" t="s">
         <v>51</v>
       </c>
-      <c r="B22" t="s">
-        <v>52</v>
-      </c>
       <c r="C22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" t="s">
         <v>55</v>
       </c>
-      <c r="D22" t="s">
-        <v>56</v>
-      </c>
       <c r="E22" t="s">
         <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" t="s">
         <v>51</v>
       </c>
-      <c r="B23" t="s">
-        <v>52</v>
-      </c>
       <c r="C23" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" t="s">
         <v>57</v>
       </c>
-      <c r="D23" t="s">
-        <v>58</v>
-      </c>
       <c r="E23" t="s">
         <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" t="s">
         <v>59</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>60</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>61</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>62</v>
       </c>
-      <c r="E24" t="s">
-        <v>63</v>
-      </c>
       <c r="F24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" t="s">
         <v>64</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>65</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>66</v>
       </c>
-      <c r="D25" t="s">
-        <v>67</v>
-      </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" t="s">
         <v>68</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>69</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>70</v>
       </c>
-      <c r="D26" t="s">
-        <v>71</v>
-      </c>
       <c r="E26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" t="s">
         <v>72</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>73</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>74</v>
       </c>
-      <c r="D27" t="s">
-        <v>75</v>
-      </c>
       <c r="E27" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" t="s">
         <v>76</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>77</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>78</v>
       </c>
-      <c r="D28" t="s">
-        <v>79</v>
-      </c>
       <c r="E28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" t="s">
         <v>80</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>81</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>82</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>83</v>
       </c>
-      <c r="E29" t="s">
-        <v>84</v>
-      </c>
       <c r="F29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" t="s">
         <v>80</v>
       </c>
-      <c r="B30" t="s">
-        <v>81</v>
-      </c>
       <c r="C30" t="s">
+        <v>84</v>
+      </c>
+      <c r="D30" t="s">
         <v>85</v>
       </c>
-      <c r="D30" t="s">
-        <v>86</v>
-      </c>
       <c r="E30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" t="s">
         <v>80</v>
       </c>
-      <c r="B31" t="s">
-        <v>81</v>
-      </c>
       <c r="C31" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" t="s">
         <v>87</v>
       </c>
-      <c r="D31" t="s">
-        <v>88</v>
-      </c>
       <c r="E31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" t="s">
         <v>80</v>
       </c>
-      <c r="B32" t="s">
-        <v>81</v>
-      </c>
       <c r="C32" t="s">
+        <v>88</v>
+      </c>
+      <c r="D32" t="s">
         <v>89</v>
       </c>
-      <c r="D32" t="s">
-        <v>90</v>
-      </c>
       <c r="E32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F32" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s">
         <v>80</v>
       </c>
-      <c r="B33" t="s">
-        <v>81</v>
-      </c>
       <c r="C33" t="s">
+        <v>90</v>
+      </c>
+      <c r="D33" t="s">
         <v>91</v>
       </c>
-      <c r="D33" t="s">
-        <v>92</v>
-      </c>
       <c r="E33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s">
         <v>80</v>
       </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
       <c r="C34" t="s">
+        <v>92</v>
+      </c>
+      <c r="D34" t="s">
         <v>93</v>
       </c>
-      <c r="D34" t="s">
-        <v>94</v>
-      </c>
       <c r="E34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" t="s">
         <v>80</v>
       </c>
-      <c r="B35" t="s">
-        <v>81</v>
-      </c>
       <c r="C35" t="s">
+        <v>94</v>
+      </c>
+      <c r="D35" t="s">
         <v>95</v>
       </c>
-      <c r="D35" t="s">
-        <v>96</v>
-      </c>
       <c r="E35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" t="s">
         <v>80</v>
       </c>
-      <c r="B36" t="s">
-        <v>81</v>
-      </c>
       <c r="C36" t="s">
+        <v>96</v>
+      </c>
+      <c r="D36" t="s">
         <v>97</v>
       </c>
-      <c r="D36" t="s">
-        <v>98</v>
-      </c>
       <c r="E36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B37" t="s">
         <v>80</v>
       </c>
-      <c r="B37" t="s">
-        <v>81</v>
-      </c>
       <c r="C37" t="s">
+        <v>98</v>
+      </c>
+      <c r="D37" t="s">
         <v>99</v>
       </c>
-      <c r="D37" t="s">
-        <v>100</v>
-      </c>
       <c r="E37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" t="s">
         <v>80</v>
       </c>
-      <c r="B38" t="s">
-        <v>81</v>
-      </c>
       <c r="C38" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" t="s">
         <v>101</v>
       </c>
-      <c r="D38" t="s">
-        <v>102</v>
-      </c>
       <c r="E38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F38" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A2:F38 C1:F1" numberStoredAsText="1"/>
+    <ignoredError sqref="A3:F11 C1:F1 B2:C2 E2:F2 A13:F38 B12:F12" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>